<commit_message>
add 'immune signature', issue https://github.com/vaccineontology/VO/issues/845
</commit_message>
<xml_diff>
--- a/src/vo_new_terms_IDs.xlsx
+++ b/src/vo_new_terms_IDs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiezhen/Documents/Ontology/VO/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{479FC3A5-F191-CD4B-BBA2-5BF7E2B1F186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D7548C8-FA63-5248-8E5F-889599887203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6120" yWindow="1860" windowWidth="20680" windowHeight="13000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9480" yWindow="1760" windowWidth="20680" windowHeight="13000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VO IDs range" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="531">
   <si>
     <t>vaccine adjuvant</t>
   </si>
@@ -1618,13 +1618,22 @@
   </si>
   <si>
     <t>ID assigned to ajuvants</t>
+  </si>
+  <si>
+    <t>immune signature</t>
+  </si>
+  <si>
+    <t>Other kinds new terms</t>
+  </si>
+  <si>
+    <t>VO:0010504</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="33" x14ac:knownFonts="1">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1862,6 +1871,12 @@
       <name val="Aptos Display"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="37">
@@ -2232,7 +2247,7 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2262,6 +2277,9 @@
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="45">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2692,7 +2710,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="13" t="s">
-        <v>21</v>
+        <v>530</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -2926,27 +2944,37 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{382F4F77-36EB-FB4D-9816-70F16A92F51F}">
-  <dimension ref="A1:B259"/>
+  <dimension ref="A1:F259"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.33203125" style="19" customWidth="1"/>
     <col min="2" max="2" width="30.1640625" style="19" customWidth="1"/>
+    <col min="5" max="5" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="E1" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="20" t="s">
         <v>22</v>
       </c>
       <c r="B2" s="21" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="E2" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="21" t="s">
         <v>23</v>
       </c>
@@ -2954,7 +2982,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="21" t="s">
         <v>24</v>
       </c>
@@ -2962,7 +2990,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="21" t="s">
         <v>25</v>
       </c>
@@ -2970,7 +2998,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="21" t="s">
         <v>470</v>
       </c>
@@ -2978,7 +3006,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="20" t="s">
         <v>26</v>
       </c>
@@ -2986,7 +3014,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="21" t="s">
         <v>27</v>
       </c>
@@ -2994,7 +3022,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="20" t="s">
         <v>28</v>
       </c>
@@ -3002,7 +3030,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
         <v>29</v>
       </c>
@@ -3010,7 +3038,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="20" t="s">
         <v>30</v>
       </c>
@@ -3018,7 +3046,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="20" t="s">
         <v>31</v>
       </c>
@@ -3026,7 +3054,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="21" t="s">
         <v>32</v>
       </c>
@@ -3034,7 +3062,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="20" t="s">
         <v>33</v>
       </c>
@@ -3042,7 +3070,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="20" t="s">
         <v>34</v>
       </c>
@@ -3050,7 +3078,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="21" t="s">
         <v>35</v>
       </c>

</xml_diff>

<commit_message>
add a drug brand name
</commit_message>
<xml_diff>
--- a/src/vo_new_terms_IDs.xlsx
+++ b/src/vo_new_terms_IDs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiezhen/Documents/Ontology/VO/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79FD4CAA-3AF0-7F4F-B386-908C6F8984FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1060A5C0-7578-ED4C-89D0-F33D8F1DB081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6200" yWindow="2360" windowWidth="24200" windowHeight="13000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2560" yWindow="3640" windowWidth="24200" windowHeight="13000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VO IDs range" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="551">
   <si>
     <t>vaccine adjuvant</t>
   </si>
@@ -1626,9 +1626,6 @@
     <t>VO:0010504</t>
   </si>
   <si>
-    <t>Assign new ID for new VO classes</t>
-  </si>
-  <si>
     <t>Assign new ID for new VO annotation or object properties</t>
   </si>
   <si>
@@ -1651,6 +1648,45 @@
   </si>
   <si>
     <t>macrophage vaccine antigen processing and presentation</t>
+  </si>
+  <si>
+    <t>VO:0010507</t>
+  </si>
+  <si>
+    <t>VO:0010508</t>
+  </si>
+  <si>
+    <t>VO:0010509</t>
+  </si>
+  <si>
+    <t>VO:0010510</t>
+  </si>
+  <si>
+    <t>VO:0010511</t>
+  </si>
+  <si>
+    <t>VO:0010512</t>
+  </si>
+  <si>
+    <t>VO:0010513</t>
+  </si>
+  <si>
+    <t>VO:0010514</t>
+  </si>
+  <si>
+    <t>VO:0010515</t>
+  </si>
+  <si>
+    <t>Assign new ID for new VO classes/instances</t>
+  </si>
+  <si>
+    <t>CAPVAXIVE</t>
+  </si>
+  <si>
+    <t>capsular polysaccharide vaccine role</t>
+  </si>
+  <si>
+    <t>polysaccharide vaccine role</t>
   </si>
 </sst>
 </file>
@@ -2301,10 +2337,8 @@
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="45">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2730,22 +2764,22 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>530</v>
+        <v>547</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="13" t="s">
-        <v>529</v>
+        <v>541</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="13" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -2984,7 +3018,9 @@
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
     <col min="2" max="2" width="30.1640625" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="12.5" customWidth="1"/>
+    <col min="6" max="6" width="52.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -2995,7 +3031,7 @@
         <v>528</v>
       </c>
       <c r="H1" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -3011,7 +3047,7 @@
       <c r="F2" t="s">
         <v>527</v>
       </c>
-      <c r="H2" s="23"/>
+      <c r="H2" s="22"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
@@ -3023,8 +3059,8 @@
       <c r="E3" t="s">
         <v>529</v>
       </c>
-      <c r="F3" s="24" t="s">
-        <v>534</v>
+      <c r="F3" s="23" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -3035,10 +3071,10 @@
         <v>259</v>
       </c>
       <c r="E4" t="s">
+        <v>534</v>
+      </c>
+      <c r="F4" s="23" t="s">
         <v>535</v>
-      </c>
-      <c r="F4" s="24" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -3049,10 +3085,10 @@
         <v>260</v>
       </c>
       <c r="E5" t="s">
+        <v>536</v>
+      </c>
+      <c r="F5" s="23" t="s">
         <v>537</v>
-      </c>
-      <c r="F5" s="24" t="s">
-        <v>538</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -3062,6 +3098,15 @@
       <c r="B6" s="20" t="s">
         <v>470</v>
       </c>
+      <c r="D6" s="24">
+        <v>46184</v>
+      </c>
+      <c r="E6" t="s">
+        <v>538</v>
+      </c>
+      <c r="F6" t="s">
+        <v>550</v>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="19" t="s">
@@ -3070,6 +3115,15 @@
       <c r="B7" s="20" t="s">
         <v>261</v>
       </c>
+      <c r="D7" s="24">
+        <v>46184</v>
+      </c>
+      <c r="E7" t="s">
+        <v>539</v>
+      </c>
+      <c r="F7" t="s">
+        <v>549</v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
@@ -3078,6 +3132,15 @@
       <c r="B8" s="20" t="s">
         <v>262</v>
       </c>
+      <c r="D8" s="24">
+        <v>46184</v>
+      </c>
+      <c r="E8" t="s">
+        <v>540</v>
+      </c>
+      <c r="F8" t="s">
+        <v>548</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="19" t="s">
@@ -3086,6 +3149,9 @@
       <c r="B9" s="20" t="s">
         <v>263</v>
       </c>
+      <c r="E9" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="19" t="s">
@@ -3094,6 +3160,9 @@
       <c r="B10" s="20" t="s">
         <v>264</v>
       </c>
+      <c r="E10" t="s">
+        <v>542</v>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="19" t="s">
@@ -3102,6 +3171,9 @@
       <c r="B11" s="20" t="s">
         <v>265</v>
       </c>
+      <c r="E11" t="s">
+        <v>543</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="19" t="s">
@@ -3110,6 +3182,9 @@
       <c r="B12" s="20" t="s">
         <v>266</v>
       </c>
+      <c r="E12" t="s">
+        <v>544</v>
+      </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="20" t="s">
@@ -3118,6 +3193,9 @@
       <c r="B13" s="20" t="s">
         <v>267</v>
       </c>
+      <c r="E13" t="s">
+        <v>545</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="19" t="s">
@@ -3126,6 +3204,9 @@
       <c r="B14" s="20" t="s">
         <v>268</v>
       </c>
+      <c r="E14" t="s">
+        <v>546</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="19" t="s">
@@ -5068,6 +5149,7 @@
       <c r="A259" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="21" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add categories and missing vaccine types
</commit_message>
<xml_diff>
--- a/src/vo_new_terms_IDs.xlsx
+++ b/src/vo_new_terms_IDs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiezhen/Documents/Ontology/VO/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1060A5C0-7578-ED4C-89D0-F33D8F1DB081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3344D0B3-238F-EF40-9019-2FC57EC901C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2560" yWindow="3640" windowWidth="24200" windowHeight="13000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6040" yWindow="800" windowWidth="24200" windowHeight="13000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VO IDs range" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="556">
   <si>
     <t>vaccine adjuvant</t>
   </si>
@@ -1687,6 +1687,21 @@
   </si>
   <si>
     <t>polysaccharide vaccine role</t>
+  </si>
+  <si>
+    <t>lipopolysaccharide vaccine role</t>
+  </si>
+  <si>
+    <t>Streptococcus pneumoniae DNA vaccine</t>
+  </si>
+  <si>
+    <t>Streptococcus pneumoniae conjugate vaccine</t>
+  </si>
+  <si>
+    <t>Streptococcus pneumoniae recombinant vector vaccine</t>
+  </si>
+  <si>
+    <t>Streptococcus pneumoniae subunit vaccine</t>
   </si>
 </sst>
 </file>
@@ -2307,7 +2322,7 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2337,7 +2352,6 @@
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="45">
@@ -2769,7 +2783,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="13" t="s">
-        <v>541</v>
+        <v>546</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -3059,7 +3073,7 @@
       <c r="E3" t="s">
         <v>529</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" t="s">
         <v>533</v>
       </c>
     </row>
@@ -3073,7 +3087,7 @@
       <c r="E4" t="s">
         <v>534</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" t="s">
         <v>535</v>
       </c>
     </row>
@@ -3087,7 +3101,7 @@
       <c r="E5" t="s">
         <v>536</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" t="s">
         <v>537</v>
       </c>
     </row>
@@ -3098,7 +3112,7 @@
       <c r="B6" s="20" t="s">
         <v>470</v>
       </c>
-      <c r="D6" s="24">
+      <c r="D6" s="23">
         <v>46184</v>
       </c>
       <c r="E6" t="s">
@@ -3115,7 +3129,7 @@
       <c r="B7" s="20" t="s">
         <v>261</v>
       </c>
-      <c r="D7" s="24">
+      <c r="D7" s="23">
         <v>46184</v>
       </c>
       <c r="E7" t="s">
@@ -3132,7 +3146,7 @@
       <c r="B8" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="23">
         <v>46184</v>
       </c>
       <c r="E8" t="s">
@@ -3149,8 +3163,14 @@
       <c r="B9" s="20" t="s">
         <v>263</v>
       </c>
+      <c r="D9" s="23">
+        <v>46184</v>
+      </c>
       <c r="E9" t="s">
         <v>541</v>
+      </c>
+      <c r="F9" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -3160,8 +3180,14 @@
       <c r="B10" s="20" t="s">
         <v>264</v>
       </c>
+      <c r="D10" s="23">
+        <v>46184</v>
+      </c>
       <c r="E10" t="s">
         <v>542</v>
+      </c>
+      <c r="F10" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -3171,8 +3197,14 @@
       <c r="B11" s="20" t="s">
         <v>265</v>
       </c>
+      <c r="D11" s="23">
+        <v>46184</v>
+      </c>
       <c r="E11" t="s">
         <v>543</v>
+      </c>
+      <c r="F11" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -3182,8 +3214,14 @@
       <c r="B12" s="20" t="s">
         <v>266</v>
       </c>
+      <c r="D12" s="23">
+        <v>46184</v>
+      </c>
       <c r="E12" t="s">
         <v>544</v>
+      </c>
+      <c r="F12" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -3193,8 +3231,14 @@
       <c r="B13" s="20" t="s">
         <v>267</v>
       </c>
+      <c r="D13" s="23">
+        <v>46184</v>
+      </c>
       <c r="E13" t="s">
         <v>545</v>
+      </c>
+      <c r="F13" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -5151,5 +5195,6 @@
   </sheetData>
   <phoneticPr fontId="21" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>